<commit_message>
update with physical activity correction
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-Tsuru.xlsx
+++ b/baseline/data_processing_elements-Tsuru.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AFCF401-7A6E-4324-BE13-5A613DB64945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFEB897C-5D9A-4892-A68C-09189895326C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{4973CF88-E30E-43C6-ADC1-EE1C260FA671}"/>
   </bookViews>
@@ -1222,7 +1222,7 @@
     <t>case_when( is.na(y24q17_1_day) &amp; is.na(y24q17_2_day) &amp; is.na(y24q17_3_day) &amp; is.na(y24q17_1_hour) &amp; is.na(y24q17_2_hour) &amp; is.na(y24q17_3_hour) &amp; is.na(y24q17_1_min) &amp; is.na(y24q17_2_min) &amp; is.na(y24q17_3_min) ~ NA;
 y24q17_1_day&gt;0 | y24q17_2_day &gt; 0 | y24q17_3_day &gt; 0 ~ 1L;
 y24q17_1_hour &gt; 0 | y24q17_2_hour &gt; 0 | y24q17_3_hour &gt; 0 ~ 1L;
-y24q17_1_min &gt; 15 | y24q17_2_min &gt; 15 | y24q17_3_min &gt; 15 ~ 1L;
+y24q17_1_min &gt;= 15 | y24q17_2_min &gt;= 15 | y24q17_3_min &gt;= 15 ~ 1L;
 ELSE ~ 0L)</t>
   </si>
 </sst>
@@ -2090,7 +2090,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" ht="30" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2128,7 +2128,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="105" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" ht="60" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2172,7 +2172,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="90" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" ht="60" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="105" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2383,7 +2383,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="105" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2503,7 +2503,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:23" ht="105" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2766,7 +2766,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:23" ht="90" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3146,7 +3146,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="39" spans="1:23" ht="90" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3222,7 +3222,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="41" spans="1:23" ht="90" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:23" ht="45" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -3336,7 +3336,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:23" ht="135" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:23" ht="120" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -3380,7 +3380,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="45" spans="1:23" ht="120" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:23" ht="105" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="46" spans="1:23" ht="90" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:23" ht="30" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -3500,7 +3500,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="48" spans="1:23" ht="150" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:23" ht="105" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -4193,7 +4193,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="66" spans="1:23" ht="210" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:23" ht="105" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -4269,7 +4269,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="68" spans="1:23" ht="225" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:23" ht="135" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -4307,7 +4307,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="69" spans="1:23" ht="75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:23" ht="30" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -4345,7 +4345,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="70" spans="1:23" ht="210" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:23" ht="105" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -4383,7 +4383,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="71" spans="1:23" ht="210" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:23" ht="105" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -4421,7 +4421,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="72" spans="1:23" ht="210" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:23" ht="105" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -4459,7 +4459,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="73" spans="1:23" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:23" ht="330" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -4497,7 +4497,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="74" spans="1:23" ht="150" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:23" ht="75" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -4535,7 +4535,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="75" spans="1:23" ht="165" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:23" ht="75" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -4696,7 +4696,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="79" spans="1:23" ht="255" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:23" ht="120" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>

</xml_diff>

<commit_message>
Correct input variable for the ID
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-Tsuru.xlsx
+++ b/baseline/data_processing_elements-Tsuru.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFEB897C-5D9A-4892-A68C-09189895326C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C26F4CA4-520F-4E25-AFF6-78726D2E3554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{4973CF88-E30E-43C6-ADC1-EE1C260FA671}"/>
   </bookViews>
@@ -1706,7 +1706,7 @@
         <v>27</v>
       </c>
       <c r="J2" t="s">
-        <v>28</v>
+        <v>349</v>
       </c>
       <c r="T2" t="s">
         <v>43</v>

</xml_diff>